<commit_message>
feat: generate codebase analysis metadata and Odoo development knowledge base files
</commit_message>
<xml_diff>
--- a/_bmad-output/Tài liệu/Chi Phí/Chi phí .xlsx
+++ b/_bmad-output/Tài liệu/Chi Phí/Chi phí .xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Odoo\bmad-odoo\_bmad-output\Tài liệu\Chi Phí\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5FE5EEB-74AD-4141-8A33-EE752A261408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B128A5-775C-4DB5-BFEC-2EF244C7034B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MH - TT - HT" sheetId="1" state="hidden" r:id="rId1"/>
@@ -1472,7 +1472,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="d\.m"/>
+    <numFmt numFmtId="164" formatCode="d\.m"/>
   </numFmts>
   <fonts count="17">
     <font>
@@ -1710,7 +1710,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1890,7 +1890,7 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -12774,7 +12774,7 @@
       <c r="AL47" s="43"/>
       <c r="AM47" s="43"/>
     </row>
-    <row r="48" spans="1:39" ht="25.9" hidden="1">
+    <row r="48" spans="1:39" ht="38.65" hidden="1">
       <c r="A48" s="41" t="s">
         <v>141</v>
       </c>
@@ -13131,7 +13131,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="59" spans="1:43" ht="115.15" hidden="1">
+    <row r="59" spans="1:43" ht="127.9" hidden="1">
       <c r="A59" s="41"/>
       <c r="B59" s="43" t="s">
         <v>142</v>
@@ -13197,7 +13197,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="61" spans="1:43" ht="38.65" hidden="1">
+    <row r="61" spans="1:43" ht="51.4" hidden="1">
       <c r="A61" s="41"/>
       <c r="B61" s="43" t="s">
         <v>142</v>
@@ -13261,7 +13261,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="63" spans="1:43" ht="51.4" hidden="1">
+    <row r="63" spans="1:43" ht="64.150000000000006" hidden="1">
       <c r="A63" s="41"/>
       <c r="B63" s="43" t="s">
         <v>142</v>
@@ -13487,7 +13487,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="70" spans="1:39" ht="51.4" hidden="1">
+    <row r="70" spans="1:39" ht="64.150000000000006" hidden="1">
       <c r="A70" s="41"/>
       <c r="B70" s="43" t="s">
         <v>142</v>

</xml_diff>